<commit_message>
Added Acceptance Tests and Color Match Themes
Implemented acceptance tests for all features in the product
 backlog, ensuring each feature has clear criteria for success.
 Also, added color match themes to the Excel files for better
 visual organization and clarity.
</commit_message>
<xml_diff>
--- a/documentation/Project Product Backlog.xlsx
+++ b/documentation/Project Product Backlog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28528"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lanthorr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jb00645\Desktop\Dev\DevOps_Project_Portfolio_Hub_Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DD06201-721F-40F7-B001-FEE609E159AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD3508B-4FE1-4E29-A52D-3025FAD68399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="0" windowWidth="19200" windowHeight="15400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -141,7 +141,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,7 +150,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -159,12 +159,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -172,16 +178,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,14 +516,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.5703125" customWidth="1"/>
-    <col min="4" max="4" width="77.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.54296875" customWidth="1"/>
+    <col min="4" max="4" width="77.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -480,203 +533,203 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="10">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="9">
         <v>1</v>
       </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="10">
         <v>1</v>
       </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="9">
         <v>1</v>
       </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="10">
         <v>2</v>
       </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="9">
         <v>2</v>
       </c>
-      <c r="B8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="10">
         <v>2</v>
       </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
         <v>2</v>
       </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="10">
         <v>3</v>
       </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
         <v>3</v>
       </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="A13">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="10">
         <v>3</v>
       </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A14">
-        <v>4</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="2" t="s">
+    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9">
+        <v>4</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15">
-        <v>4</v>
-      </c>
-      <c r="B15" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="2" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="10">
+        <v>4</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="8" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Wireframe for Project Pages and Page Flow
Drew a wireframe for the project's UI design, featuring 6 pages and a navigation bar.
 The wireframe illustrates how users will flow between pages and includes a chart
 indicating whether the user needs to be logged in or out to view each page.
</commit_message>
<xml_diff>
--- a/documentation/Project Product Backlog.xlsx
+++ b/documentation/Project Product Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jb00645\Desktop\Dev\DevOps_Project_Portfolio_Hub_Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD3508B-4FE1-4E29-A52D-3025FAD68399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA1A2B8-F714-4971-BBBC-A3448880E300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="0" windowWidth="19200" windowHeight="15400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12540" yWindow="11670" windowWidth="14640" windowHeight="9270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>